<commit_message>
update on 06/21 by sudharsan
</commit_message>
<xml_diff>
--- a/data/interim/new-bills-parsed/Profile5000_pivoted.xlsx
+++ b/data/interim/new-bills-parsed/Profile5000_pivoted.xlsx
@@ -106,9 +106,6 @@
     <t>Rider CCR</t>
   </si>
   <si>
-    <t>Rider CE kW</t>
-  </si>
-  <si>
     <t>Rider CE kWh</t>
   </si>
   <si>
@@ -136,6 +133,9 @@
     <t>Rider GV kWh</t>
   </si>
   <si>
+    <t>Rider GV kw</t>
+  </si>
+  <si>
     <t>Rider OSW KW</t>
   </si>
   <si>
@@ -1525,6 +1525,42 @@
     <t>$19.68</t>
   </si>
   <si>
+    <t>$64.85</t>
+  </si>
+  <si>
+    <t>$88.68</t>
+  </si>
+  <si>
+    <t>$96.79</t>
+  </si>
+  <si>
+    <t>$77.12</t>
+  </si>
+  <si>
+    <t>$44.78</t>
+  </si>
+  <si>
+    <t>$49.19</t>
+  </si>
+  <si>
+    <t>$24.95</t>
+  </si>
+  <si>
+    <t>$39.31</t>
+  </si>
+  <si>
+    <t>$34.84</t>
+  </si>
+  <si>
+    <t>$25.93</t>
+  </si>
+  <si>
+    <t>$23.56</t>
+  </si>
+  <si>
+    <t>$26.51</t>
+  </si>
+  <si>
     <t>$37.25</t>
   </si>
   <si>
@@ -1549,42 +1585,6 @@
     <t>$42.97</t>
   </si>
   <si>
-    <t>$64.85</t>
-  </si>
-  <si>
-    <t>$88.68</t>
-  </si>
-  <si>
-    <t>$96.79</t>
-  </si>
-  <si>
-    <t>$77.12</t>
-  </si>
-  <si>
-    <t>$44.78</t>
-  </si>
-  <si>
-    <t>$49.19</t>
-  </si>
-  <si>
-    <t>$24.95</t>
-  </si>
-  <si>
-    <t>$39.31</t>
-  </si>
-  <si>
-    <t>$34.84</t>
-  </si>
-  <si>
-    <t>$25.93</t>
-  </si>
-  <si>
-    <t>$23.56</t>
-  </si>
-  <si>
-    <t>$26.51</t>
-  </si>
-  <si>
     <t>$35.36</t>
   </si>
   <si>
@@ -1807,6 +1807,30 @@
     <t>$66.57</t>
   </si>
   <si>
+    <t>$53.04</t>
+  </si>
+  <si>
+    <t>$72.52</t>
+  </si>
+  <si>
+    <t>$79.15</t>
+  </si>
+  <si>
+    <t>$63.07</t>
+  </si>
+  <si>
+    <t>$36.62</t>
+  </si>
+  <si>
+    <t>$40.22</t>
+  </si>
+  <si>
+    <t>$20.40</t>
+  </si>
+  <si>
+    <t>$29.39</t>
+  </si>
+  <si>
     <t>$54.78</t>
   </si>
   <si>
@@ -1835,30 +1859,6 @@
   </si>
   <si>
     <t>$43.57</t>
-  </si>
-  <si>
-    <t>$53.04</t>
-  </si>
-  <si>
-    <t>$72.52</t>
-  </si>
-  <si>
-    <t>$79.15</t>
-  </si>
-  <si>
-    <t>$63.07</t>
-  </si>
-  <si>
-    <t>$36.62</t>
-  </si>
-  <si>
-    <t>$40.22</t>
-  </si>
-  <si>
-    <t>$20.40</t>
-  </si>
-  <si>
-    <t>$29.39</t>
   </si>
   <si>
     <t>$41.49</t>
@@ -3050,8 +3050,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -3067,7 +3075,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -3075,12 +3083,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3379,235 +3405,235 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:77">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="AY1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BA1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BB1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BC1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BD1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BE1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BF1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BG1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BH1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BI1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BJ1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BK1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BL1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BM1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BN1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BO1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BP1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BQ1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BR1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="BS1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="BT1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="BU1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="BV1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="BW1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="BX1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="BY1" s="1" t="s">
         <v>76</v>
       </c>
     </row>
@@ -3681,16 +3707,16 @@
       <c r="AD2" t="s">
         <v>471</v>
       </c>
-      <c r="AE2" t="s">
-        <v>503</v>
-      </c>
-      <c r="AI2" t="s">
+      <c r="AF2" t="s">
+        <v>515</v>
+      </c>
+      <c r="AH2" t="s">
         <v>538</v>
       </c>
+      <c r="AK2" t="s">
+        <v>572</v>
+      </c>
       <c r="AL2" t="s">
-        <v>572</v>
-      </c>
-      <c r="AM2" t="s">
         <v>589</v>
       </c>
       <c r="AO2" t="s">
@@ -3824,16 +3850,16 @@
       <c r="AD3" t="s">
         <v>472</v>
       </c>
-      <c r="AE3" t="s">
-        <v>504</v>
-      </c>
-      <c r="AI3" t="s">
+      <c r="AF3" t="s">
+        <v>516</v>
+      </c>
+      <c r="AH3" t="s">
         <v>539</v>
       </c>
+      <c r="AK3" t="s">
+        <v>573</v>
+      </c>
       <c r="AL3" t="s">
-        <v>573</v>
-      </c>
-      <c r="AM3" t="s">
         <v>590</v>
       </c>
       <c r="AO3" t="s">
@@ -3964,16 +3990,16 @@
       <c r="AD4" t="s">
         <v>473</v>
       </c>
-      <c r="AE4" t="s">
-        <v>505</v>
-      </c>
-      <c r="AI4" t="s">
+      <c r="AF4" t="s">
+        <v>517</v>
+      </c>
+      <c r="AH4" t="s">
         <v>540</v>
       </c>
+      <c r="AK4" t="s">
+        <v>574</v>
+      </c>
       <c r="AL4" t="s">
-        <v>574</v>
-      </c>
-      <c r="AM4" t="s">
         <v>591</v>
       </c>
       <c r="AO4" t="s">
@@ -4104,16 +4130,16 @@
       <c r="AD5" t="s">
         <v>474</v>
       </c>
-      <c r="AE5" t="s">
-        <v>506</v>
-      </c>
-      <c r="AI5" t="s">
+      <c r="AF5" t="s">
+        <v>518</v>
+      </c>
+      <c r="AH5" t="s">
         <v>541</v>
       </c>
+      <c r="AK5" t="s">
+        <v>575</v>
+      </c>
       <c r="AL5" t="s">
-        <v>575</v>
-      </c>
-      <c r="AM5" t="s">
         <v>592</v>
       </c>
       <c r="AO5" t="s">
@@ -4244,16 +4270,16 @@
       <c r="AD6" t="s">
         <v>475</v>
       </c>
-      <c r="AE6" t="s">
-        <v>507</v>
-      </c>
-      <c r="AI6" t="s">
+      <c r="AF6" t="s">
+        <v>519</v>
+      </c>
+      <c r="AH6" t="s">
         <v>542</v>
       </c>
+      <c r="AK6" t="s">
+        <v>576</v>
+      </c>
       <c r="AL6" t="s">
-        <v>576</v>
-      </c>
-      <c r="AM6" t="s">
         <v>593</v>
       </c>
       <c r="AO6" t="s">
@@ -4387,16 +4413,16 @@
       <c r="AD7" t="s">
         <v>476</v>
       </c>
-      <c r="AE7" t="s">
-        <v>508</v>
-      </c>
-      <c r="AI7" t="s">
+      <c r="AF7" t="s">
+        <v>520</v>
+      </c>
+      <c r="AH7" t="s">
         <v>543</v>
       </c>
+      <c r="AK7" t="s">
+        <v>577</v>
+      </c>
       <c r="AL7" t="s">
-        <v>577</v>
-      </c>
-      <c r="AM7" t="s">
         <v>594</v>
       </c>
       <c r="AO7" t="s">
@@ -4527,16 +4553,16 @@
       <c r="AD8" t="s">
         <v>477</v>
       </c>
-      <c r="AE8" t="s">
-        <v>507</v>
-      </c>
-      <c r="AI8" t="s">
+      <c r="AF8" t="s">
+        <v>519</v>
+      </c>
+      <c r="AH8" t="s">
         <v>542</v>
       </c>
+      <c r="AK8" t="s">
+        <v>576</v>
+      </c>
       <c r="AL8" t="s">
-        <v>576</v>
-      </c>
-      <c r="AM8" t="s">
         <v>593</v>
       </c>
       <c r="AO8" t="s">
@@ -4667,16 +4693,16 @@
       <c r="AD9" t="s">
         <v>478</v>
       </c>
-      <c r="AE9" t="s">
-        <v>509</v>
-      </c>
-      <c r="AI9" t="s">
+      <c r="AF9" t="s">
+        <v>521</v>
+      </c>
+      <c r="AH9" t="s">
         <v>544</v>
       </c>
+      <c r="AK9" t="s">
+        <v>578</v>
+      </c>
       <c r="AL9" t="s">
-        <v>578</v>
-      </c>
-      <c r="AM9" t="s">
         <v>595</v>
       </c>
       <c r="AO9" t="s">
@@ -4807,16 +4833,16 @@
       <c r="AD10" t="s">
         <v>479</v>
       </c>
-      <c r="AE10" t="s">
-        <v>510</v>
-      </c>
-      <c r="AI10" t="s">
+      <c r="AF10" t="s">
+        <v>522</v>
+      </c>
+      <c r="AH10" t="s">
         <v>545</v>
       </c>
+      <c r="AK10" t="s">
+        <v>579</v>
+      </c>
       <c r="AL10" t="s">
-        <v>579</v>
-      </c>
-      <c r="AM10" t="s">
         <v>596</v>
       </c>
       <c r="AO10" t="s">
@@ -4947,17 +4973,17 @@
       <c r="AD11" t="s">
         <v>480</v>
       </c>
-      <c r="AG11" t="s">
+      <c r="AF11" t="s">
         <v>523</v>
       </c>
-      <c r="AI11" t="s">
+      <c r="AH11" t="s">
         <v>546</v>
       </c>
-      <c r="AL11" t="s">
+      <c r="AK11" t="s">
         <v>580</v>
       </c>
-      <c r="AM11" t="s">
-        <v>597</v>
+      <c r="AN11" t="s">
+        <v>605</v>
       </c>
       <c r="AO11" t="s">
         <v>623</v>
@@ -5090,17 +5116,17 @@
       <c r="AD12" t="s">
         <v>481</v>
       </c>
-      <c r="AG12" t="s">
+      <c r="AF12" t="s">
         <v>524</v>
       </c>
-      <c r="AI12" t="s">
+      <c r="AH12" t="s">
         <v>547</v>
       </c>
-      <c r="AL12" t="s">
+      <c r="AK12" t="s">
         <v>581</v>
       </c>
-      <c r="AM12" t="s">
-        <v>598</v>
+      <c r="AN12" t="s">
+        <v>606</v>
       </c>
       <c r="AO12" t="s">
         <v>624</v>
@@ -5230,17 +5256,17 @@
       <c r="AD13" t="s">
         <v>482</v>
       </c>
-      <c r="AG13" t="s">
+      <c r="AF13" t="s">
         <v>525</v>
       </c>
-      <c r="AI13" t="s">
+      <c r="AH13" t="s">
         <v>548</v>
       </c>
-      <c r="AL13" t="s">
+      <c r="AK13" t="s">
         <v>582</v>
       </c>
-      <c r="AM13" t="s">
-        <v>599</v>
+      <c r="AN13" t="s">
+        <v>607</v>
       </c>
       <c r="AO13" t="s">
         <v>625</v>
@@ -5370,17 +5396,17 @@
       <c r="AD14" t="s">
         <v>483</v>
       </c>
-      <c r="AG14" t="s">
+      <c r="AF14" t="s">
         <v>526</v>
       </c>
-      <c r="AI14" t="s">
+      <c r="AH14" t="s">
         <v>549</v>
       </c>
-      <c r="AL14" t="s">
+      <c r="AK14" t="s">
         <v>583</v>
       </c>
-      <c r="AM14" t="s">
-        <v>600</v>
+      <c r="AN14" t="s">
+        <v>608</v>
       </c>
       <c r="AO14" t="s">
         <v>626</v>
@@ -5510,16 +5536,16 @@
       <c r="AD15" t="s">
         <v>484</v>
       </c>
-      <c r="AG15" t="s">
-        <v>507</v>
-      </c>
-      <c r="AI15" t="s">
+      <c r="AF15" t="s">
+        <v>519</v>
+      </c>
+      <c r="AH15" t="s">
         <v>542</v>
       </c>
-      <c r="AL15" t="s">
+      <c r="AK15" t="s">
         <v>576</v>
       </c>
-      <c r="AM15" t="s">
+      <c r="AN15" t="s">
         <v>593</v>
       </c>
       <c r="AO15" t="s">
@@ -5653,17 +5679,17 @@
       <c r="AD16" t="s">
         <v>485</v>
       </c>
-      <c r="AG16" t="s">
+      <c r="AF16" t="s">
         <v>527</v>
       </c>
-      <c r="AI16" t="s">
+      <c r="AH16" t="s">
         <v>550</v>
       </c>
-      <c r="AL16" t="s">
+      <c r="AK16" t="s">
         <v>584</v>
       </c>
-      <c r="AM16" t="s">
-        <v>601</v>
+      <c r="AN16" t="s">
+        <v>609</v>
       </c>
       <c r="AO16" t="s">
         <v>627</v>
@@ -5793,17 +5819,17 @@
       <c r="AD17" t="s">
         <v>486</v>
       </c>
-      <c r="AG17" t="s">
+      <c r="AF17" t="s">
         <v>528</v>
       </c>
-      <c r="AI17" t="s">
+      <c r="AH17" t="s">
         <v>551</v>
       </c>
-      <c r="AL17" t="s">
+      <c r="AK17" t="s">
         <v>132</v>
       </c>
-      <c r="AM17" t="s">
-        <v>602</v>
+      <c r="AN17" t="s">
+        <v>610</v>
       </c>
       <c r="AO17" t="s">
         <v>628</v>
@@ -5933,17 +5959,17 @@
       <c r="AD18" t="s">
         <v>487</v>
       </c>
-      <c r="AG18" t="s">
+      <c r="AF18" t="s">
         <v>529</v>
       </c>
-      <c r="AI18" t="s">
+      <c r="AH18" t="s">
         <v>552</v>
       </c>
-      <c r="AL18" t="s">
+      <c r="AK18" t="s">
         <v>585</v>
       </c>
-      <c r="AM18" t="s">
-        <v>603</v>
+      <c r="AN18" t="s">
+        <v>611</v>
       </c>
       <c r="AO18" t="s">
         <v>629</v>
@@ -6073,17 +6099,17 @@
       <c r="AD19" t="s">
         <v>488</v>
       </c>
-      <c r="AG19" t="s">
+      <c r="AF19" t="s">
         <v>530</v>
       </c>
-      <c r="AI19" t="s">
+      <c r="AH19" t="s">
         <v>553</v>
       </c>
-      <c r="AL19" t="s">
+      <c r="AK19" t="s">
         <v>586</v>
       </c>
-      <c r="AM19" t="s">
-        <v>604</v>
+      <c r="AN19" t="s">
+        <v>612</v>
       </c>
       <c r="AO19" t="s">
         <v>630</v>
@@ -6213,17 +6239,17 @@
       <c r="AD20" t="s">
         <v>489</v>
       </c>
-      <c r="AG20" t="s">
+      <c r="AF20" t="s">
         <v>531</v>
       </c>
-      <c r="AI20" t="s">
+      <c r="AH20" t="s">
         <v>554</v>
       </c>
-      <c r="AL20" t="s">
+      <c r="AK20" t="s">
         <v>587</v>
       </c>
-      <c r="AM20" t="s">
-        <v>605</v>
+      <c r="AN20" t="s">
+        <v>613</v>
       </c>
       <c r="AO20" t="s">
         <v>631</v>
@@ -6356,17 +6382,17 @@
       <c r="AD21" t="s">
         <v>490</v>
       </c>
-      <c r="AG21" t="s">
+      <c r="AF21" t="s">
         <v>532</v>
       </c>
-      <c r="AI21" t="s">
+      <c r="AH21" t="s">
         <v>555</v>
       </c>
-      <c r="AL21" t="s">
+      <c r="AK21" t="s">
         <v>588</v>
       </c>
-      <c r="AM21" t="s">
-        <v>606</v>
+      <c r="AN21" t="s">
+        <v>614</v>
       </c>
       <c r="AO21" t="s">
         <v>632</v>
@@ -6493,14 +6519,14 @@
       <c r="AD22" t="s">
         <v>491</v>
       </c>
-      <c r="AF22" t="s">
-        <v>511</v>
-      </c>
-      <c r="AJ22" t="s">
+      <c r="AE22" t="s">
+        <v>503</v>
+      </c>
+      <c r="AI22" t="s">
         <v>556</v>
       </c>
-      <c r="AN22" t="s">
-        <v>607</v>
+      <c r="AM22" t="s">
+        <v>597</v>
       </c>
       <c r="AP22" t="s">
         <v>633</v>
@@ -6624,14 +6650,14 @@
       <c r="AD23" t="s">
         <v>492</v>
       </c>
-      <c r="AF23" t="s">
-        <v>512</v>
-      </c>
-      <c r="AJ23" t="s">
+      <c r="AE23" t="s">
+        <v>504</v>
+      </c>
+      <c r="AI23" t="s">
         <v>557</v>
       </c>
-      <c r="AN23" t="s">
-        <v>608</v>
+      <c r="AM23" t="s">
+        <v>598</v>
       </c>
       <c r="AP23" t="s">
         <v>634</v>
@@ -6755,14 +6781,14 @@
       <c r="AD24" t="s">
         <v>493</v>
       </c>
-      <c r="AF24" t="s">
-        <v>513</v>
-      </c>
-      <c r="AJ24" t="s">
+      <c r="AE24" t="s">
+        <v>505</v>
+      </c>
+      <c r="AI24" t="s">
         <v>558</v>
       </c>
-      <c r="AN24" t="s">
-        <v>609</v>
+      <c r="AM24" t="s">
+        <v>599</v>
       </c>
       <c r="AP24" t="s">
         <v>635</v>
@@ -6886,14 +6912,14 @@
       <c r="AD25" t="s">
         <v>494</v>
       </c>
-      <c r="AF25" t="s">
-        <v>514</v>
-      </c>
-      <c r="AJ25" t="s">
+      <c r="AE25" t="s">
+        <v>506</v>
+      </c>
+      <c r="AI25" t="s">
         <v>559</v>
       </c>
-      <c r="AN25" t="s">
-        <v>610</v>
+      <c r="AM25" t="s">
+        <v>600</v>
       </c>
       <c r="AP25" t="s">
         <v>636</v>
@@ -7014,14 +7040,14 @@
       <c r="AD26" t="s">
         <v>495</v>
       </c>
-      <c r="AF26" t="s">
-        <v>515</v>
-      </c>
-      <c r="AJ26" t="s">
+      <c r="AE26" t="s">
+        <v>507</v>
+      </c>
+      <c r="AI26" t="s">
         <v>560</v>
       </c>
-      <c r="AN26" t="s">
-        <v>611</v>
+      <c r="AM26" t="s">
+        <v>601</v>
       </c>
       <c r="AP26" t="s">
         <v>637</v>
@@ -7142,14 +7168,14 @@
       <c r="AD27" t="s">
         <v>496</v>
       </c>
-      <c r="AF27" t="s">
-        <v>516</v>
-      </c>
-      <c r="AJ27" t="s">
+      <c r="AE27" t="s">
+        <v>508</v>
+      </c>
+      <c r="AI27" t="s">
         <v>467</v>
       </c>
-      <c r="AN27" t="s">
-        <v>612</v>
+      <c r="AM27" t="s">
+        <v>602</v>
       </c>
       <c r="AP27" t="s">
         <v>638</v>
@@ -7273,17 +7299,17 @@
       <c r="AD28" t="s">
         <v>497</v>
       </c>
-      <c r="AF28" t="s">
-        <v>517</v>
-      </c>
-      <c r="AH28" t="s">
-        <v>444</v>
-      </c>
-      <c r="AJ28" t="s">
+      <c r="AE28" t="s">
+        <v>509</v>
+      </c>
+      <c r="AG28" t="s">
+        <v>444</v>
+      </c>
+      <c r="AI28" t="s">
         <v>561</v>
       </c>
-      <c r="AN28" t="s">
-        <v>613</v>
+      <c r="AM28" t="s">
+        <v>603</v>
       </c>
       <c r="AP28" t="s">
         <v>639</v>
@@ -7407,20 +7433,20 @@
       <c r="AD29" t="s">
         <v>498</v>
       </c>
-      <c r="AF29" t="s">
-        <v>518</v>
-      </c>
-      <c r="AH29" t="s">
+      <c r="AE29" t="s">
+        <v>510</v>
+      </c>
+      <c r="AG29" t="s">
         <v>533</v>
       </c>
+      <c r="AI29" t="s">
+        <v>562</v>
+      </c>
       <c r="AJ29" t="s">
-        <v>562</v>
-      </c>
-      <c r="AK29" t="s">
         <v>567</v>
       </c>
-      <c r="AN29" t="s">
-        <v>614</v>
+      <c r="AM29" t="s">
+        <v>604</v>
       </c>
       <c r="AP29" t="s">
         <v>640</v>
@@ -7544,19 +7570,19 @@
       <c r="AD30" t="s">
         <v>499</v>
       </c>
-      <c r="AF30" t="s">
-        <v>519</v>
-      </c>
-      <c r="AH30" t="s">
+      <c r="AE30" t="s">
+        <v>511</v>
+      </c>
+      <c r="AG30" t="s">
         <v>534</v>
       </c>
+      <c r="AI30" t="s">
+        <v>563</v>
+      </c>
       <c r="AJ30" t="s">
-        <v>563</v>
-      </c>
-      <c r="AK30" t="s">
         <v>568</v>
       </c>
-      <c r="AN30" t="s">
+      <c r="AM30" t="s">
         <v>444</v>
       </c>
       <c r="AP30" t="s">
@@ -7681,19 +7707,19 @@
       <c r="AD31" t="s">
         <v>500</v>
       </c>
-      <c r="AF31" t="s">
-        <v>520</v>
-      </c>
-      <c r="AH31" t="s">
+      <c r="AE31" t="s">
+        <v>512</v>
+      </c>
+      <c r="AG31" t="s">
         <v>535</v>
       </c>
+      <c r="AI31" t="s">
+        <v>564</v>
+      </c>
       <c r="AJ31" t="s">
-        <v>564</v>
-      </c>
-      <c r="AK31" t="s">
         <v>569</v>
       </c>
-      <c r="AN31" t="s">
+      <c r="AM31" t="s">
         <v>444</v>
       </c>
       <c r="AP31" t="s">
@@ -7818,19 +7844,19 @@
       <c r="AD32" t="s">
         <v>501</v>
       </c>
-      <c r="AF32" t="s">
-        <v>521</v>
-      </c>
-      <c r="AH32" t="s">
+      <c r="AE32" t="s">
+        <v>513</v>
+      </c>
+      <c r="AG32" t="s">
         <v>536</v>
       </c>
+      <c r="AI32" t="s">
+        <v>565</v>
+      </c>
       <c r="AJ32" t="s">
-        <v>565</v>
-      </c>
-      <c r="AK32" t="s">
         <v>570</v>
       </c>
-      <c r="AN32" t="s">
+      <c r="AM32" t="s">
         <v>444</v>
       </c>
       <c r="AP32" t="s">
@@ -7958,19 +7984,19 @@
       <c r="AD33" t="s">
         <v>502</v>
       </c>
-      <c r="AF33" t="s">
-        <v>522</v>
-      </c>
-      <c r="AH33" t="s">
+      <c r="AE33" t="s">
+        <v>514</v>
+      </c>
+      <c r="AG33" t="s">
         <v>537</v>
       </c>
+      <c r="AI33" t="s">
+        <v>566</v>
+      </c>
       <c r="AJ33" t="s">
-        <v>566</v>
-      </c>
-      <c r="AK33" t="s">
         <v>571</v>
       </c>
-      <c r="AN33" t="s">
+      <c r="AM33" t="s">
         <v>444</v>
       </c>
       <c r="AP33" t="s">

</xml_diff>